<commit_message>
update role and keanggotaan
add upload
</commit_message>
<xml_diff>
--- a/public/document/Keanggotaan Tim Template.xlsx
+++ b/public/document/Keanggotaan Tim Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rifqind\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F452126-3584-46B5-8E0C-2489107A88EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C24B6538-E0DD-4554-9939-8A2070A15868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4C485BC0-E57A-4123-BC42-163A0E71FB7D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>nama_tim</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>(nama tim harus sesuai dengan yang ada di sistem)</t>
-  </si>
-  <si>
-    <t>(nama pegawai harus sesuai dengan yang ada di sistem)</t>
   </si>
   <si>
     <r>
@@ -80,6 +77,15 @@
       </rPr>
       <t>)</t>
     </r>
+  </si>
+  <si>
+    <t>nip_(lama atau baru)</t>
+  </si>
+  <si>
+    <t>(masukkan nip atau nama pegawai)</t>
+  </si>
+  <si>
+    <t>(masukkan nama_pegawai atau nip, nama pegawai harus sesuai dengan yang ada di sistem)</t>
   </si>
 </sst>
 </file>
@@ -129,10 +135,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,34 +478,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C736A5-242B-4FAC-9B78-72E82FDE845A}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.21875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="22" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="35.21875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>